<commit_message>
feat: improve color image previews and automate submission style rules
</commit_message>
<xml_diff>
--- a/docs/送审输入模板.xlsx
+++ b/docs/送审输入模板.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品资料" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="商品资料" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,17 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,20 +448,15 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>上下装</t>
+          <t>面料</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>面料</t>
+          <t>成本</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>成本</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
         <is>
           <t>图片</t>
         </is>

</xml_diff>